<commit_message>
Atualização automática - 17/08/2026 12:00
</commit_message>
<xml_diff>
--- a/Aplicativos/consumo/consumo.xlsx
+++ b/Aplicativos/consumo/consumo.xlsx
@@ -1,10 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4507"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="27932"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\usr\Downloads\Equipes_Agentes\Aplicativos\consumo\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{603DF377-F2FD-4ABE-B995-C6B5ED65436E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="16380" windowHeight="8190" tabRatio="278"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="278" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ajuste" sheetId="5" r:id="rId1"/>
@@ -13,11 +19,16 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">ajuste!$A$1:$C$316</definedName>
   </definedNames>
   <calcPr calcId="125725"/>
+  <extLst>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="318" uniqueCount="315">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="326" uniqueCount="323">
   <si>
     <t xml:space="preserve">PRANCHETA DURATEX </t>
   </si>
@@ -962,13 +973,37 @@
   </si>
   <si>
     <t>descricao consinco</t>
+  </si>
+  <si>
+    <t>CONS SACO PP RAMINHO 17X45</t>
+  </si>
+  <si>
+    <t>CONS FITA ADESIVA 12X30MM CRISTAL</t>
+  </si>
+  <si>
+    <t>CONS ETQ COUCHE 100X50 55MM GREEN</t>
+  </si>
+  <si>
+    <t>CONS ETIQUETA LARANJA DATA DE VALID</t>
+  </si>
+  <si>
+    <t>CONS ETIQ LINGUICA M PIMENTAO ALEG</t>
+  </si>
+  <si>
+    <t>CONS ETIQ LING FRANGO ALEGRETE</t>
+  </si>
+  <si>
+    <t>CONS ETIQ COUCHE 100X50 53MM RED</t>
+  </si>
+  <si>
+    <t>CONS EMB DC650 POTE QUAD C 300</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="5">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -1164,6 +1199,14 @@
       <rgbColor rgb="00333333"/>
     </indexedColors>
   </colors>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -1514,9 +1557,9 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C316"/>
-  <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="12.75"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:C324"/>
+  <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10.85546875" style="3" customWidth="1"/>
     <col min="2" max="2" width="50.85546875" style="3" bestFit="1" customWidth="1"/>
@@ -1524,7 +1567,7 @@
     <col min="4" max="16384" width="11.5703125" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" s="12" customFormat="1" ht="15">
+    <row r="1" spans="1:3" s="12" customFormat="1" ht="15" x14ac:dyDescent="0.25">
       <c r="A1" s="14" t="s">
         <v>313</v>
       </c>
@@ -1535,7 +1578,7 @@
         <v>292</v>
       </c>
     </row>
-    <row r="2" spans="1:3" s="6" customFormat="1">
+    <row r="2" spans="1:3" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A2" s="5">
         <v>35394</v>
       </c>
@@ -1546,7 +1589,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A3" s="3">
         <v>36108</v>
       </c>
@@ -1557,7 +1600,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A4" s="3">
         <v>35375</v>
       </c>
@@ -1568,7 +1611,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A5" s="3">
         <v>35438</v>
       </c>
@@ -1579,7 +1622,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A6" s="3">
         <v>35554</v>
       </c>
@@ -1590,7 +1633,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A7" s="3">
         <v>35798</v>
       </c>
@@ -1601,7 +1644,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A8" s="3">
         <v>35937</v>
       </c>
@@ -1612,7 +1655,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:3">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A9" s="3">
         <v>35773</v>
       </c>
@@ -1623,7 +1666,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:3">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A10" s="3">
         <v>36068</v>
       </c>
@@ -1634,7 +1677,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:3">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A11" s="3">
         <v>36088</v>
       </c>
@@ -1645,7 +1688,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:3">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A12" s="3">
         <v>36089</v>
       </c>
@@ -1656,7 +1699,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:3">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A13" s="3">
         <v>36091</v>
       </c>
@@ -1667,7 +1710,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:3">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A14" s="3">
         <v>35640</v>
       </c>
@@ -1678,7 +1721,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:3">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A15" s="3">
         <v>35742</v>
       </c>
@@ -1689,7 +1732,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:3">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A16" s="3">
         <v>35775</v>
       </c>
@@ -1700,7 +1743,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:3">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A17" s="3">
         <v>36093</v>
       </c>
@@ -1711,7 +1754,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="1:3">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A18" s="3">
         <v>36096</v>
       </c>
@@ -1722,7 +1765,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:3">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A19" s="3">
         <v>36163</v>
       </c>
@@ -1733,7 +1776,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="1:3">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A20" s="3">
         <v>35372</v>
       </c>
@@ -1744,7 +1787,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="21" spans="1:3">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A21" s="3">
         <v>35440</v>
       </c>
@@ -1755,7 +1798,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="1:3">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A22" s="3">
         <v>1234501</v>
       </c>
@@ -1766,7 +1809,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="23" spans="1:3">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A23" s="3">
         <v>36098</v>
       </c>
@@ -1777,7 +1820,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="1:3">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A24" s="3">
         <v>35363</v>
       </c>
@@ -1788,7 +1831,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="1:3">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A25" s="3">
         <v>35380</v>
       </c>
@@ -1799,7 +1842,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="26" spans="1:3">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A26" s="3">
         <v>35935</v>
       </c>
@@ -1810,7 +1853,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="27" spans="1:3">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A27" s="3">
         <v>35368</v>
       </c>
@@ -1821,7 +1864,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="28" spans="1:3">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A28" s="3">
         <v>35920</v>
       </c>
@@ -1832,7 +1875,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="29" spans="1:3">
+    <row r="29" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A29" s="3">
         <v>35924</v>
       </c>
@@ -1843,7 +1886,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="30" spans="1:3">
+    <row r="30" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A30" s="3">
         <v>35987</v>
       </c>
@@ -1854,7 +1897,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="31" spans="1:3">
+    <row r="31" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A31" s="3">
         <v>35986</v>
       </c>
@@ -1865,7 +1908,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="32" spans="1:3">
+    <row r="32" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A32" s="3">
         <v>35642</v>
       </c>
@@ -1876,7 +1919,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="33" spans="1:3">
+    <row r="33" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A33" s="3">
         <v>35534</v>
       </c>
@@ -1887,7 +1930,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="34" spans="1:3">
+    <row r="34" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A34" s="3">
         <v>35536</v>
       </c>
@@ -1898,7 +1941,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="35" spans="1:3">
+    <row r="35" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A35" s="3">
         <v>35559</v>
       </c>
@@ -1909,7 +1952,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="36" spans="1:3">
+    <row r="36" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A36" s="3">
         <v>35555</v>
       </c>
@@ -1920,7 +1963,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="37" spans="1:3">
+    <row r="37" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A37" s="3">
         <v>35450</v>
       </c>
@@ -1931,7 +1974,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="38" spans="1:3">
+    <row r="38" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A38" s="3">
         <v>36499</v>
       </c>
@@ -1942,7 +1985,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="39" spans="1:3">
+    <row r="39" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A39" s="3">
         <v>36082</v>
       </c>
@@ -1953,7 +1996,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="40" spans="1:3">
+    <row r="40" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A40" s="3">
         <v>36139</v>
       </c>
@@ -1964,7 +2007,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="41" spans="1:3">
+    <row r="41" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A41" s="3">
         <v>35651</v>
       </c>
@@ -1975,7 +2018,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="42" spans="1:3">
+    <row r="42" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A42" s="3">
         <v>36102</v>
       </c>
@@ -1986,7 +2029,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="43" spans="1:3">
+    <row r="43" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A43" s="3">
         <v>36109</v>
       </c>
@@ -1997,7 +2040,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="44" spans="1:3">
+    <row r="44" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A44" s="3">
         <v>36095</v>
       </c>
@@ -2008,7 +2051,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="45" spans="1:3">
+    <row r="45" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A45" s="3">
         <v>35529</v>
       </c>
@@ -2019,7 +2062,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="46" spans="1:3">
+    <row r="46" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A46" s="3">
         <v>35530</v>
       </c>
@@ -2030,7 +2073,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="47" spans="1:3">
+    <row r="47" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A47" s="3">
         <v>35531</v>
       </c>
@@ -2041,7 +2084,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="48" spans="1:3">
+    <row r="48" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A48" s="3">
         <v>35523</v>
       </c>
@@ -2052,7 +2095,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="49" spans="1:3">
+    <row r="49" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A49" s="3">
         <v>36097</v>
       </c>
@@ -2063,7 +2106,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="50" spans="1:3" ht="14.25">
+    <row r="50" spans="1:3" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A50" s="3">
         <v>35517</v>
       </c>
@@ -2074,7 +2117,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="51" spans="1:3">
+    <row r="51" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A51" s="3">
         <v>35355</v>
       </c>
@@ -2085,7 +2128,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="52" spans="1:3">
+    <row r="52" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A52" s="3">
         <v>35373</v>
       </c>
@@ -2096,7 +2139,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="53" spans="1:3">
+    <row r="53" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A53" s="3">
         <v>35485</v>
       </c>
@@ -2107,7 +2150,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="54" spans="1:3">
+    <row r="54" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A54" s="3">
         <v>35489</v>
       </c>
@@ -2118,7 +2161,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="55" spans="1:3">
+    <row r="55" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A55" s="3">
         <v>35379</v>
       </c>
@@ -2129,7 +2172,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="56" spans="1:3">
+    <row r="56" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A56" s="3">
         <v>35737</v>
       </c>
@@ -2140,7 +2183,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="57" spans="1:3">
+    <row r="57" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A57" s="3">
         <v>35359</v>
       </c>
@@ -2151,7 +2194,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="58" spans="1:3">
+    <row r="58" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A58" s="3">
         <v>35377</v>
       </c>
@@ -2162,7 +2205,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="59" spans="1:3">
+    <row r="59" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A59" s="3">
         <v>36520</v>
       </c>
@@ -2173,7 +2216,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="60" spans="1:3">
+    <row r="60" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A60" s="3">
         <v>35360</v>
       </c>
@@ -2184,7 +2227,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="61" spans="1:3">
+    <row r="61" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A61" s="3">
         <v>60172</v>
       </c>
@@ -2195,7 +2238,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="62" spans="1:3">
+    <row r="62" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A62" s="3">
         <v>60172</v>
       </c>
@@ -2206,7 +2249,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="63" spans="1:3">
+    <row r="63" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A63" s="3">
         <v>60172</v>
       </c>
@@ -2217,7 +2260,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="64" spans="1:3">
+    <row r="64" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A64" s="3">
         <v>60172</v>
       </c>
@@ -2228,7 +2271,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="65" spans="1:3">
+    <row r="65" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A65" s="3">
         <v>38344</v>
       </c>
@@ -2239,7 +2282,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="66" spans="1:3">
+    <row r="66" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A66" s="3">
         <v>38344</v>
       </c>
@@ -2250,7 +2293,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="67" spans="1:3">
+    <row r="67" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A67" s="3">
         <v>38344</v>
       </c>
@@ -2261,7 +2304,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="68" spans="1:3">
+    <row r="68" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A68" s="3">
         <v>38344</v>
       </c>
@@ -2272,7 +2315,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="69" spans="1:3">
+    <row r="69" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A69" s="3">
         <v>38344</v>
       </c>
@@ -2283,7 +2326,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="70" spans="1:3">
+    <row r="70" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A70" s="3">
         <v>60175</v>
       </c>
@@ -2294,7 +2337,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="71" spans="1:3">
+    <row r="71" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A71" s="3">
         <v>60175</v>
       </c>
@@ -2305,7 +2348,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="72" spans="1:3">
+    <row r="72" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A72" s="3">
         <v>60175</v>
       </c>
@@ -2316,7 +2359,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="73" spans="1:3">
+    <row r="73" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A73" s="3">
         <v>60175</v>
       </c>
@@ -2327,7 +2370,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="74" spans="1:3">
+    <row r="74" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A74" s="3">
         <v>35997</v>
       </c>
@@ -2338,7 +2381,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="75" spans="1:3">
+    <row r="75" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A75" s="3">
         <v>35999</v>
       </c>
@@ -2349,7 +2392,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="76" spans="1:3">
+    <row r="76" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A76" s="3">
         <v>36034</v>
       </c>
@@ -2360,7 +2403,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="77" spans="1:3">
+    <row r="77" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A77" s="3">
         <v>36014</v>
       </c>
@@ -2371,7 +2414,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="78" spans="1:3">
+    <row r="78" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A78" s="3">
         <v>36015</v>
       </c>
@@ -2382,7 +2425,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="79" spans="1:3">
+    <row r="79" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A79" s="3">
         <v>36016</v>
       </c>
@@ -2393,7 +2436,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="80" spans="1:3">
+    <row r="80" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A80" s="3">
         <v>36044</v>
       </c>
@@ -2404,7 +2447,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="81" spans="1:3">
+    <row r="81" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A81" s="3">
         <v>36018</v>
       </c>
@@ -2415,7 +2458,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="82" spans="1:3">
+    <row r="82" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A82" s="3">
         <v>36019</v>
       </c>
@@ -2426,7 +2469,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="83" spans="1:3">
+    <row r="83" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A83" s="3">
         <v>36020</v>
       </c>
@@ -2437,7 +2480,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="84" spans="1:3">
+    <row r="84" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A84" s="3">
         <v>36022</v>
       </c>
@@ -2448,7 +2491,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="85" spans="1:3">
+    <row r="85" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A85" s="3">
         <v>36025</v>
       </c>
@@ -2459,7 +2502,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="86" spans="1:3">
+    <row r="86" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A86" s="3">
         <v>36039</v>
       </c>
@@ -2470,7 +2513,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="87" spans="1:3">
+    <row r="87" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A87" s="3">
         <v>36023</v>
       </c>
@@ -2481,7 +2524,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="88" spans="1:3">
+    <row r="88" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A88" s="3">
         <v>1234502</v>
       </c>
@@ -2492,7 +2535,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="89" spans="1:3">
+    <row r="89" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A89" s="3">
         <v>36047</v>
       </c>
@@ -2503,7 +2546,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="90" spans="1:3">
+    <row r="90" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A90" s="3">
         <v>36028</v>
       </c>
@@ -2514,7 +2557,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="91" spans="1:3">
+    <row r="91" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A91" s="3">
         <v>36045</v>
       </c>
@@ -2525,7 +2568,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="92" spans="1:3">
+    <row r="92" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A92" s="3">
         <v>36029</v>
       </c>
@@ -2536,7 +2579,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="93" spans="1:3">
+    <row r="93" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A93" s="3">
         <v>36053</v>
       </c>
@@ -2547,7 +2590,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="94" spans="1:3">
+    <row r="94" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A94" s="3">
         <v>36032</v>
       </c>
@@ -2558,7 +2601,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="95" spans="1:3">
+    <row r="95" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A95" s="3">
         <v>36045</v>
       </c>
@@ -2569,7 +2612,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="96" spans="1:3">
+    <row r="96" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A96" s="3">
         <v>1234503</v>
       </c>
@@ -2580,7 +2623,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="97" spans="1:3">
+    <row r="97" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A97" s="3">
         <v>1234504</v>
       </c>
@@ -2591,7 +2634,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="98" spans="1:3">
+    <row r="98" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A98" s="3">
         <v>36013</v>
       </c>
@@ -2602,7 +2645,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="99" spans="1:3">
+    <row r="99" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A99" s="3">
         <v>36038</v>
       </c>
@@ -2613,7 +2656,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="100" spans="1:3">
+    <row r="100" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A100" s="3">
         <v>36050</v>
       </c>
@@ -2624,7 +2667,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="101" spans="1:3">
+    <row r="101" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A101" s="3">
         <v>36050</v>
       </c>
@@ -2635,7 +2678,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="102" spans="1:3">
+    <row r="102" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A102" s="3">
         <v>36050</v>
       </c>
@@ -2646,7 +2689,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="103" spans="1:3">
+    <row r="103" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A103" s="3">
         <v>36033</v>
       </c>
@@ -2657,7 +2700,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="104" spans="1:3">
+    <row r="104" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A104" s="3">
         <v>36021</v>
       </c>
@@ -2668,7 +2711,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="105" spans="1:3">
+    <row r="105" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A105" s="3">
         <v>36024</v>
       </c>
@@ -2679,7 +2722,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="106" spans="1:3">
+    <row r="106" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A106" s="3">
         <v>36049</v>
       </c>
@@ -2690,7 +2733,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="107" spans="1:3">
+    <row r="107" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A107" s="3">
         <v>36129</v>
       </c>
@@ -2701,7 +2744,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="108" spans="1:3">
+    <row r="108" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A108" s="3">
         <v>36128</v>
       </c>
@@ -2712,7 +2755,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="109" spans="1:3">
+    <row r="109" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A109" s="3">
         <v>35494</v>
       </c>
@@ -2723,7 +2766,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="110" spans="1:3">
+    <row r="110" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A110" s="3">
         <v>35501</v>
       </c>
@@ -2734,7 +2777,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="111" spans="1:3">
+    <row r="111" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A111" s="3">
         <v>35498</v>
       </c>
@@ -2745,7 +2788,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="112" spans="1:3">
+    <row r="112" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A112" s="3">
         <v>35497</v>
       </c>
@@ -2756,7 +2799,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="113" spans="1:3">
+    <row r="113" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A113" s="3">
         <v>35495</v>
       </c>
@@ -2767,7 +2810,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="114" spans="1:3">
+    <row r="114" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A114" s="3">
         <v>35503</v>
       </c>
@@ -2778,7 +2821,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="115" spans="1:3">
+    <row r="115" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A115" s="3">
         <v>35993</v>
       </c>
@@ -2789,7 +2832,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="116" spans="1:3">
+    <row r="116" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A116" s="3">
         <v>35995</v>
       </c>
@@ -2800,7 +2843,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="117" spans="1:3">
+    <row r="117" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A117" s="3">
         <v>35367</v>
       </c>
@@ -2811,7 +2854,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="118" spans="1:3">
+    <row r="118" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A118" s="3">
         <v>35525</v>
       </c>
@@ -2822,7 +2865,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="119" spans="1:3">
+    <row r="119" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A119" s="3">
         <v>35471</v>
       </c>
@@ -2833,7 +2876,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="120" spans="1:3">
+    <row r="120" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A120" s="3">
         <v>35474</v>
       </c>
@@ -2844,7 +2887,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="121" spans="1:3">
+    <row r="121" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A121" s="3">
         <v>37285</v>
       </c>
@@ -2855,7 +2898,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="122" spans="1:3">
+    <row r="122" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A122" s="3">
         <v>35364</v>
       </c>
@@ -2866,7 +2909,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="123" spans="1:3">
+    <row r="123" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A123" s="3">
         <v>35755</v>
       </c>
@@ -2877,7 +2920,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="124" spans="1:3">
+    <row r="124" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A124" s="3">
         <v>35772</v>
       </c>
@@ -2888,7 +2931,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="125" spans="1:3">
+    <row r="125" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A125" s="3">
         <v>35718</v>
       </c>
@@ -2899,7 +2942,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="126" spans="1:3">
+    <row r="126" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A126" s="3">
         <v>35451</v>
       </c>
@@ -2910,7 +2953,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="127" spans="1:3">
+    <row r="127" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A127" s="3">
         <v>36623</v>
       </c>
@@ -2921,7 +2964,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="128" spans="1:3">
+    <row r="128" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A128" s="3">
         <v>35659</v>
       </c>
@@ -2932,7 +2975,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="129" spans="1:3">
+    <row r="129" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A129" s="3">
         <v>36649</v>
       </c>
@@ -2943,7 +2986,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="130" spans="1:3">
+    <row r="130" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A130" s="3">
         <v>36648</v>
       </c>
@@ -2954,7 +2997,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="131" spans="1:3">
+    <row r="131" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A131" s="3">
         <v>35686</v>
       </c>
@@ -2965,7 +3008,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="132" spans="1:3">
+    <row r="132" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A132" s="3">
         <v>37581</v>
       </c>
@@ -2976,7 +3019,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="133" spans="1:3">
+    <row r="133" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A133" s="3">
         <v>35454</v>
       </c>
@@ -2987,7 +3030,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="134" spans="1:3">
+    <row r="134" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A134" s="3">
         <v>1234505</v>
       </c>
@@ -2998,7 +3041,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="135" spans="1:3">
+    <row r="135" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A135" s="3">
         <v>1234506</v>
       </c>
@@ -3009,7 +3052,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="136" spans="1:3">
+    <row r="136" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A136" s="3">
         <v>36144</v>
       </c>
@@ -3020,7 +3063,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="137" spans="1:3">
+    <row r="137" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A137" s="3">
         <v>35980</v>
       </c>
@@ -3031,7 +3074,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="138" spans="1:3">
+    <row r="138" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A138" s="3">
         <v>36142</v>
       </c>
@@ -3042,7 +3085,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="139" spans="1:3">
+    <row r="139" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A139" s="3">
         <v>35405</v>
       </c>
@@ -3053,7 +3096,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="140" spans="1:3">
+    <row r="140" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A140" s="3">
         <v>35499</v>
       </c>
@@ -3064,7 +3107,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="141" spans="1:3">
+    <row r="141" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A141" s="3">
         <v>35362</v>
       </c>
@@ -3075,7 +3118,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="142" spans="1:3">
+    <row r="142" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A142" s="3">
         <v>1234507</v>
       </c>
@@ -3086,7 +3129,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="143" spans="1:3">
+    <row r="143" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A143" s="3">
         <v>35746</v>
       </c>
@@ -3097,7 +3140,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="144" spans="1:3">
+    <row r="144" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A144" s="3">
         <v>35745</v>
       </c>
@@ -3108,7 +3151,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="145" spans="1:3">
+    <row r="145" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A145" s="3">
         <v>37598</v>
       </c>
@@ -3119,7 +3162,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="146" spans="1:3">
+    <row r="146" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A146" s="3">
         <v>35396</v>
       </c>
@@ -3130,7 +3173,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="147" spans="1:3">
+    <row r="147" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A147" s="3">
         <v>35500</v>
       </c>
@@ -3141,7 +3184,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="148" spans="1:3">
+    <row r="148" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A148" s="3">
         <v>35382</v>
       </c>
@@ -3152,7 +3195,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="149" spans="1:3">
+    <row r="149" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A149" s="3">
         <v>35358</v>
       </c>
@@ -3163,7 +3206,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="150" spans="1:3">
+    <row r="150" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A150" s="3">
         <v>35390</v>
       </c>
@@ -3174,7 +3217,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="151" spans="1:3">
+    <row r="151" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A151" s="3">
         <v>36151</v>
       </c>
@@ -3185,7 +3228,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="152" spans="1:3">
+    <row r="152" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A152" s="3">
         <v>36149</v>
       </c>
@@ -3196,7 +3239,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="153" spans="1:3">
+    <row r="153" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A153" s="3">
         <v>35957</v>
       </c>
@@ -3207,7 +3250,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="154" spans="1:3">
+    <row r="154" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A154" s="3">
         <v>35958</v>
       </c>
@@ -3218,7 +3261,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="155" spans="1:3" s="6" customFormat="1">
+    <row r="155" spans="1:3" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A155" s="6">
         <v>35461</v>
       </c>
@@ -3229,7 +3272,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="156" spans="1:3" ht="13.5" customHeight="1">
+    <row r="156" spans="1:3" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A156" s="3">
         <v>35465</v>
       </c>
@@ -3240,7 +3283,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="157" spans="1:3">
+    <row r="157" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A157" s="3">
         <v>35461</v>
       </c>
@@ -3251,7 +3294,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="158" spans="1:3">
+    <row r="158" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A158" s="3">
         <v>1234508</v>
       </c>
@@ -3262,7 +3305,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="159" spans="1:3">
+    <row r="159" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A159" s="3">
         <v>1234509</v>
       </c>
@@ -3273,7 +3316,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="160" spans="1:3">
+    <row r="160" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A160" s="3">
         <v>1234510</v>
       </c>
@@ -3284,7 +3327,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="161" spans="1:3">
+    <row r="161" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A161" s="3">
         <v>1234511</v>
       </c>
@@ -3295,7 +3338,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="162" spans="1:3">
+    <row r="162" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A162" s="3">
         <v>1234512</v>
       </c>
@@ -3306,7 +3349,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="163" spans="1:3">
+    <row r="163" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A163" s="3">
         <v>1234513</v>
       </c>
@@ -3317,7 +3360,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="164" spans="1:3">
+    <row r="164" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A164" s="3">
         <v>35447</v>
       </c>
@@ -3328,7 +3371,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="165" spans="1:3">
+    <row r="165" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A165" s="3">
         <v>35428</v>
       </c>
@@ -3339,7 +3382,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="166" spans="1:3">
+    <row r="166" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A166" s="3">
         <v>35427</v>
       </c>
@@ -3350,7 +3393,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="167" spans="1:3">
+    <row r="167" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A167" s="3">
         <v>35425</v>
       </c>
@@ -3361,7 +3404,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="168" spans="1:3" s="6" customFormat="1">
+    <row r="168" spans="1:3" s="6" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A168" s="6">
         <v>35433</v>
       </c>
@@ -3372,7 +3415,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="169" spans="1:3">
+    <row r="169" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A169" s="3">
         <v>35457</v>
       </c>
@@ -3383,7 +3426,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="170" spans="1:3">
+    <row r="170" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A170" s="3">
         <v>35460</v>
       </c>
@@ -3394,7 +3437,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="171" spans="1:3">
+    <row r="171" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A171" s="3">
         <v>35456</v>
       </c>
@@ -3405,7 +3448,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="172" spans="1:3">
+    <row r="172" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A172" s="3">
         <v>35437</v>
       </c>
@@ -3416,7 +3459,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="173" spans="1:3" s="10" customFormat="1">
+    <row r="173" spans="1:3" s="10" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A173" s="10">
         <v>35434</v>
       </c>
@@ -3427,7 +3470,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="174" spans="1:3" s="10" customFormat="1">
+    <row r="174" spans="1:3" s="10" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A174" s="10">
         <v>36517</v>
       </c>
@@ -3438,7 +3481,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="175" spans="1:3">
+    <row r="175" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A175" s="3">
         <v>35433</v>
       </c>
@@ -3449,7 +3492,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="176" spans="1:3">
+    <row r="176" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A176" s="3">
         <v>35513</v>
       </c>
@@ -3460,7 +3503,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="177" spans="1:3">
+    <row r="177" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A177" s="3">
         <v>35515</v>
       </c>
@@ -3471,7 +3514,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="178" spans="1:3">
+    <row r="178" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A178" s="3">
         <v>35510</v>
       </c>
@@ -3482,7 +3525,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="179" spans="1:3">
+    <row r="179" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A179" s="3">
         <v>35516</v>
       </c>
@@ -3493,7 +3536,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="180" spans="1:3">
+    <row r="180" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A180" s="3">
         <v>35436</v>
       </c>
@@ -3504,7 +3547,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="181" spans="1:3">
+    <row r="181" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A181" s="3">
         <v>35432</v>
       </c>
@@ -3515,7 +3558,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="182" spans="1:3">
+    <row r="182" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A182" s="3">
         <v>35435</v>
       </c>
@@ -3526,7 +3569,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="183" spans="1:3">
+    <row r="183" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A183" s="3">
         <v>35374</v>
       </c>
@@ -3537,7 +3580,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="184" spans="1:3">
+    <row r="184" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A184" s="3">
         <v>35370</v>
       </c>
@@ -3548,7 +3591,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="185" spans="1:3">
+    <row r="185" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A185" s="3">
         <v>1234514</v>
       </c>
@@ -3559,7 +3602,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="186" spans="1:3">
+    <row r="186" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A186" s="3">
         <v>35371</v>
       </c>
@@ -3570,7 +3613,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="187" spans="1:3">
+    <row r="187" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A187" s="3">
         <v>1234515</v>
       </c>
@@ -3581,7 +3624,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="188" spans="1:3">
+    <row r="188" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A188" s="3">
         <v>36147</v>
       </c>
@@ -3592,7 +3635,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="189" spans="1:3" s="4" customFormat="1">
+    <row r="189" spans="1:3" s="4" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A189" s="7">
         <v>38490</v>
       </c>
@@ -3603,7 +3646,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="190" spans="1:3">
+    <row r="190" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A190" s="3">
         <v>36054</v>
       </c>
@@ -3614,7 +3657,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="191" spans="1:3">
+    <row r="191" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A191" s="3">
         <v>1234516</v>
       </c>
@@ -3625,7 +3668,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="192" spans="1:3">
+    <row r="192" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A192" s="3">
         <v>36126</v>
       </c>
@@ -3636,7 +3679,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="193" spans="1:3">
+    <row r="193" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A193" s="3">
         <v>36125</v>
       </c>
@@ -3647,7 +3690,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="194" spans="1:3">
+    <row r="194" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A194" s="3">
         <v>36127</v>
       </c>
@@ -3658,7 +3701,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="195" spans="1:3">
+    <row r="195" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A195" s="3">
         <v>36054</v>
       </c>
@@ -3669,7 +3712,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="196" spans="1:3">
+    <row r="196" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A196" s="3">
         <v>1234517</v>
       </c>
@@ -3680,7 +3723,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="197" spans="1:3">
+    <row r="197" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A197" s="3">
         <v>35400</v>
       </c>
@@ -3691,7 +3734,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="198" spans="1:3">
+    <row r="198" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A198" s="3">
         <v>35786</v>
       </c>
@@ -3702,7 +3745,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="199" spans="1:3">
+    <row r="199" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A199" s="3">
         <v>35381</v>
       </c>
@@ -3713,7 +3756,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="200" spans="1:3">
+    <row r="200" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A200" s="3">
         <v>35381</v>
       </c>
@@ -3724,7 +3767,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="201" spans="1:3">
+    <row r="201" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A201" s="3">
         <v>35392</v>
       </c>
@@ -3735,7 +3778,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="202" spans="1:3">
+    <row r="202" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A202" s="3">
         <v>36124</v>
       </c>
@@ -3746,7 +3789,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="203" spans="1:3">
+    <row r="203" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A203" s="3">
         <v>38488</v>
       </c>
@@ -3757,7 +3800,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="204" spans="1:3">
+    <row r="204" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A204" s="3">
         <v>35482</v>
       </c>
@@ -3768,7 +3811,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="205" spans="1:3">
+    <row r="205" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A205" s="3">
         <v>35771</v>
       </c>
@@ -3779,7 +3822,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="206" spans="1:3">
+    <row r="206" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A206" s="3">
         <v>35386</v>
       </c>
@@ -3790,7 +3833,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="207" spans="1:3">
+    <row r="207" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A207" s="3">
         <v>36118</v>
       </c>
@@ -3801,7 +3844,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="208" spans="1:3">
+    <row r="208" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A208" s="3">
         <v>36119</v>
       </c>
@@ -3812,7 +3855,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="209" spans="1:3">
+    <row r="209" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A209" s="3">
         <v>36120</v>
       </c>
@@ -3823,7 +3866,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="210" spans="1:3">
+    <row r="210" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A210" s="3">
         <v>36121</v>
       </c>
@@ -3834,7 +3877,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="211" spans="1:3">
+    <row r="211" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A211" s="3">
         <v>36135</v>
       </c>
@@ -3845,7 +3888,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="212" spans="1:3">
+    <row r="212" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A212" s="3">
         <v>36136</v>
       </c>
@@ -3856,7 +3899,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="213" spans="1:3">
+    <row r="213" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A213" s="3">
         <v>36070</v>
       </c>
@@ -3867,7 +3910,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="214" spans="1:3">
+    <row r="214" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A214" s="3">
         <v>1234518</v>
       </c>
@@ -3878,7 +3921,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="215" spans="1:3">
+    <row r="215" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A215" s="3">
         <v>35439</v>
       </c>
@@ -3889,7 +3932,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="216" spans="1:3">
+    <row r="216" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A216" s="3">
         <v>35605</v>
       </c>
@@ -3900,7 +3943,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="217" spans="1:3">
+    <row r="217" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A217" s="3">
         <v>35983</v>
       </c>
@@ -3911,7 +3954,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="218" spans="1:3">
+    <row r="218" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A218" s="3">
         <v>1234519</v>
       </c>
@@ -3922,7 +3965,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="219" spans="1:3">
+    <row r="219" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A219" s="3">
         <v>1234520</v>
       </c>
@@ -3933,7 +3976,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="220" spans="1:3">
+    <row r="220" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A220" s="3">
         <v>36160</v>
       </c>
@@ -3944,7 +3987,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="221" spans="1:3">
+    <row r="221" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A221" s="3">
         <v>36158</v>
       </c>
@@ -3955,7 +3998,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="222" spans="1:3">
+    <row r="222" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A222" s="3">
         <v>36162</v>
       </c>
@@ -3966,7 +4009,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="223" spans="1:3">
+    <row r="223" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A223" s="3">
         <v>35532</v>
       </c>
@@ -3977,7 +4020,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="224" spans="1:3">
+    <row r="224" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A224" s="3">
         <v>38489</v>
       </c>
@@ -3988,7 +4031,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="225" spans="1:3">
+    <row r="225" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A225" s="3">
         <v>1234521</v>
       </c>
@@ -3999,7 +4042,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="226" spans="1:3">
+    <row r="226" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A226" s="3">
         <v>36516</v>
       </c>
@@ -4010,7 +4053,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="227" spans="1:3">
+    <row r="227" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A227" s="3">
         <v>38491</v>
       </c>
@@ -4021,7 +4064,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="228" spans="1:3">
+    <row r="228" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A228" s="3">
         <v>36716</v>
       </c>
@@ -4032,7 +4075,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="229" spans="1:3">
+    <row r="229" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A229" s="3">
         <v>35404</v>
       </c>
@@ -4043,7 +4086,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="230" spans="1:3" ht="13.5" customHeight="1">
+    <row r="230" spans="1:3" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A230" s="3">
         <v>1234522</v>
       </c>
@@ -4054,7 +4097,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="231" spans="1:3">
+    <row r="231" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A231" s="3">
         <v>1234523</v>
       </c>
@@ -4065,7 +4108,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="232" spans="1:3">
+    <row r="232" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A232" s="3">
         <v>35487</v>
       </c>
@@ -4076,7 +4119,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="233" spans="1:3">
+    <row r="233" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A233" s="3">
         <v>1234524</v>
       </c>
@@ -4087,7 +4130,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="234" spans="1:3">
+    <row r="234" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A234" s="3">
         <v>36066</v>
       </c>
@@ -4098,7 +4141,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="235" spans="1:3">
+    <row r="235" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A235" s="3">
         <v>1234525</v>
       </c>
@@ -4109,7 +4152,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="236" spans="1:3">
+    <row r="236" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A236" s="3">
         <v>35419</v>
       </c>
@@ -4120,7 +4163,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="237" spans="1:3">
+    <row r="237" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A237" s="3">
         <v>35424</v>
       </c>
@@ -4131,7 +4174,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="238" spans="1:3">
+    <row r="238" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A238" s="3">
         <v>35431</v>
       </c>
@@ -4142,7 +4185,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="239" spans="1:3">
+    <row r="239" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A239" s="3">
         <v>35445</v>
       </c>
@@ -4153,7 +4196,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="240" spans="1:3">
+    <row r="240" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A240" s="3">
         <v>35408</v>
       </c>
@@ -4164,7 +4207,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="241" spans="1:3">
+    <row r="241" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A241" s="3">
         <v>35411</v>
       </c>
@@ -4175,7 +4218,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="242" spans="1:3">
+    <row r="242" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A242" s="3">
         <v>35415</v>
       </c>
@@ -4186,7 +4229,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="243" spans="1:3">
+    <row r="243" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A243" s="3">
         <v>1234526</v>
       </c>
@@ -4197,7 +4240,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="244" spans="1:3">
+    <row r="244" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A244" s="3">
         <v>35449</v>
       </c>
@@ -4208,7 +4251,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="245" spans="1:3">
+    <row r="245" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A245" s="3">
         <v>35453</v>
       </c>
@@ -4219,7 +4262,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="246" spans="1:3">
+    <row r="246" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A246" s="3">
         <v>35952</v>
       </c>
@@ -4230,7 +4273,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="247" spans="1:3">
+    <row r="247" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A247" s="3">
         <v>37604</v>
       </c>
@@ -4241,7 +4284,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="248" spans="1:3">
+    <row r="248" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A248" s="3">
         <v>36140</v>
       </c>
@@ -4252,7 +4295,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="249" spans="1:3">
+    <row r="249" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A249" s="3">
         <v>35357</v>
       </c>
@@ -4263,7 +4306,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="250" spans="1:3">
+    <row r="250" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A250" s="3">
         <v>36123</v>
       </c>
@@ -4274,7 +4317,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="251" spans="1:3">
+    <row r="251" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A251" s="3">
         <v>35953</v>
       </c>
@@ -4285,7 +4328,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="252" spans="1:3">
+    <row r="252" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A252" s="3">
         <v>35954</v>
       </c>
@@ -4296,7 +4339,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="253" spans="1:3">
+    <row r="253" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A253" s="3">
         <v>36104</v>
       </c>
@@ -4307,7 +4350,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="254" spans="1:3">
+    <row r="254" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A254" s="3">
         <v>36105</v>
       </c>
@@ -4318,7 +4361,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="255" spans="1:3">
+    <row r="255" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A255" s="3">
         <v>36073</v>
       </c>
@@ -4329,7 +4372,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="256" spans="1:3">
+    <row r="256" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A256" s="3">
         <v>36138</v>
       </c>
@@ -4340,7 +4383,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="257" spans="1:3" s="9" customFormat="1">
+    <row r="257" spans="1:3" s="9" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A257" s="9">
         <v>35472</v>
       </c>
@@ -4351,7 +4394,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="258" spans="1:3">
+    <row r="258" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A258" s="3">
         <v>35378</v>
       </c>
@@ -4362,7 +4405,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="259" spans="1:3">
+    <row r="259" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A259" s="3">
         <v>35506</v>
       </c>
@@ -4373,7 +4416,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="260" spans="1:3">
+    <row r="260" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A260" s="3">
         <v>34738</v>
       </c>
@@ -4384,7 +4427,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="261" spans="1:3">
+    <row r="261" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A261" s="3">
         <v>35366</v>
       </c>
@@ -4395,7 +4438,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="262" spans="1:3">
+    <row r="262" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A262" s="3">
         <v>35406</v>
       </c>
@@ -4406,7 +4449,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="263" spans="1:3">
+    <row r="263" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A263" s="3">
         <v>3613</v>
       </c>
@@ -4417,7 +4460,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="264" spans="1:3">
+    <row r="264" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A264" s="3">
         <v>1234527</v>
       </c>
@@ -4428,7 +4471,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="265" spans="1:3">
+    <row r="265" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A265" s="3">
         <v>36094</v>
       </c>
@@ -4439,7 +4482,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="266" spans="1:3">
+    <row r="266" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A266" s="3">
         <v>36641</v>
       </c>
@@ -4450,7 +4493,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="267" spans="1:3">
+    <row r="267" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A267" s="3">
         <v>35858</v>
       </c>
@@ -4461,7 +4504,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="268" spans="1:3">
+    <row r="268" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A268" s="3">
         <v>35911</v>
       </c>
@@ -4472,7 +4515,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="269" spans="1:3">
+    <row r="269" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A269" s="3">
         <v>35849</v>
       </c>
@@ -4483,7 +4526,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="270" spans="1:3">
+    <row r="270" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A270" s="3">
         <v>35842</v>
       </c>
@@ -4494,7 +4537,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="271" spans="1:3">
+    <row r="271" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A271" s="3">
         <v>35810</v>
       </c>
@@ -4505,7 +4548,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="272" spans="1:3">
+    <row r="272" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A272" s="3">
         <v>35835</v>
       </c>
@@ -4516,7 +4559,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="273" spans="1:3">
+    <row r="273" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A273" s="3">
         <v>35840</v>
       </c>
@@ -4527,7 +4570,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="274" spans="1:3">
+    <row r="274" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A274" s="3">
         <v>35825</v>
       </c>
@@ -4538,7 +4581,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="275" spans="1:3">
+    <row r="275" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A275" s="3">
         <v>35814</v>
       </c>
@@ -4549,7 +4592,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="276" spans="1:3">
+    <row r="276" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A276" s="3">
         <v>35838</v>
       </c>
@@ -4560,7 +4603,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="277" spans="1:3">
+    <row r="277" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A277" s="3">
         <v>35852</v>
       </c>
@@ -4571,7 +4614,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="278" spans="1:3">
+    <row r="278" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A278" s="3">
         <v>35802</v>
       </c>
@@ -4582,7 +4625,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="279" spans="1:3">
+    <row r="279" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A279" s="3">
         <v>35812</v>
       </c>
@@ -4593,7 +4636,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="280" spans="1:3">
+    <row r="280" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A280" s="3">
         <v>35828</v>
       </c>
@@ -4604,7 +4647,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="281" spans="1:3">
+    <row r="281" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A281" s="3">
         <v>35898</v>
       </c>
@@ -4615,7 +4658,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="282" spans="1:3">
+    <row r="282" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A282" s="3">
         <v>35805</v>
       </c>
@@ -4626,7 +4669,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="283" spans="1:3">
+    <row r="283" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A283" s="3">
         <v>35888</v>
       </c>
@@ -4637,7 +4680,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="284" spans="1:3">
+    <row r="284" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A284" s="3">
         <v>35882</v>
       </c>
@@ -4648,7 +4691,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="285" spans="1:3">
+    <row r="285" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A285" s="3">
         <v>36099</v>
       </c>
@@ -4659,7 +4702,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="286" spans="1:3">
+    <row r="286" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A286" s="3">
         <v>35612</v>
       </c>
@@ -4670,7 +4713,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="287" spans="1:3">
+    <row r="287" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A287" s="3">
         <v>35619</v>
       </c>
@@ -4681,7 +4724,7 @@
         <v>250</v>
       </c>
     </row>
-    <row r="288" spans="1:3">
+    <row r="288" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A288" s="3">
         <v>35478</v>
       </c>
@@ -4692,7 +4735,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="289" spans="1:3">
+    <row r="289" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A289" s="3">
         <v>35483</v>
       </c>
@@ -4703,7 +4746,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="290" spans="1:3">
+    <row r="290" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A290" s="3">
         <v>36132</v>
       </c>
@@ -4714,7 +4757,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="291" spans="1:3">
+    <row r="291" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A291" s="3">
         <v>36130</v>
       </c>
@@ -4725,7 +4768,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="292" spans="1:3">
+    <row r="292" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A292" s="3">
         <v>36064</v>
       </c>
@@ -4736,7 +4779,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="293" spans="1:3">
+    <row r="293" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A293" s="3">
         <v>36057</v>
       </c>
@@ -4747,7 +4790,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="294" spans="1:3">
+    <row r="294" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A294" s="3">
         <v>36066</v>
       </c>
@@ -4758,7 +4801,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="295" spans="1:3">
+    <row r="295" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A295" s="3">
         <v>36061</v>
       </c>
@@ -4769,7 +4812,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="296" spans="1:3">
+    <row r="296" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A296" s="3">
         <v>36056</v>
       </c>
@@ -4780,7 +4823,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="297" spans="1:3">
+    <row r="297" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A297" s="3">
         <v>36065</v>
       </c>
@@ -4791,7 +4834,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="298" spans="1:3">
+    <row r="298" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A298" s="3">
         <v>36055</v>
       </c>
@@ -4802,7 +4845,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="299" spans="1:3">
+    <row r="299" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A299" s="3">
         <v>36058</v>
       </c>
@@ -4813,7 +4856,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="300" spans="1:3">
+    <row r="300" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A300" s="3">
         <v>36010</v>
       </c>
@@ -4824,7 +4867,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="301" spans="1:3">
+    <row r="301" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A301" s="3">
         <v>36060</v>
       </c>
@@ -4835,7 +4878,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="302" spans="1:3">
+    <row r="302" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A302" s="3">
         <v>36007</v>
       </c>
@@ -4846,7 +4889,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="303" spans="1:3">
+    <row r="303" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A303" s="3">
         <v>36001</v>
       </c>
@@ -4857,7 +4900,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="304" spans="1:3">
+    <row r="304" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A304" s="3">
         <v>36009</v>
       </c>
@@ -4868,7 +4911,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="305" spans="1:3">
+    <row r="305" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A305" s="3">
         <v>36003</v>
       </c>
@@ -4879,7 +4922,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="306" spans="1:3">
+    <row r="306" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A306" s="3">
         <v>35779</v>
       </c>
@@ -4890,7 +4933,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="307" spans="1:3">
+    <row r="307" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A307" s="3">
         <v>35540</v>
       </c>
@@ -4901,7 +4944,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="308" spans="1:3">
+    <row r="308" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A308" s="3">
         <v>36145</v>
       </c>
@@ -4912,7 +4955,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="309" spans="1:3">
+    <row r="309" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A309" s="3">
         <v>35935</v>
       </c>
@@ -4923,7 +4966,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="310" spans="1:3">
+    <row r="310" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A310" s="3">
         <v>36152</v>
       </c>
@@ -4934,7 +4977,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="311" spans="1:3">
+    <row r="311" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A311" s="3">
         <v>35738</v>
       </c>
@@ -4945,7 +4988,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="312" spans="1:3">
+    <row r="312" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A312" s="3">
         <v>37388</v>
       </c>
@@ -4956,7 +4999,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="313" spans="1:3">
+    <row r="313" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A313" s="3">
         <v>36153</v>
       </c>
@@ -4967,7 +5010,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="314" spans="1:3">
+    <row r="314" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A314" s="3">
         <v>35739</v>
       </c>
@@ -4978,7 +5021,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="315" spans="1:3">
+    <row r="315" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A315" s="3">
         <v>36154</v>
       </c>
@@ -4989,7 +5032,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="316" spans="1:3">
+    <row r="316" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A316" s="3">
         <v>35376</v>
       </c>
@@ -5000,8 +5043,96 @@
         <v>1</v>
       </c>
     </row>
+    <row r="317" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A317" s="3">
+        <v>35468</v>
+      </c>
+      <c r="B317" s="3" t="s">
+        <v>315</v>
+      </c>
+      <c r="C317" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="318" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A318" s="3">
+        <v>36076</v>
+      </c>
+      <c r="B318" s="3" t="s">
+        <v>316</v>
+      </c>
+      <c r="C318" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="319" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A319" s="3">
+        <v>36067</v>
+      </c>
+      <c r="B319" s="3" t="s">
+        <v>317</v>
+      </c>
+      <c r="C319" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="320" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A320" s="3">
+        <v>36133</v>
+      </c>
+      <c r="B320" s="3" t="s">
+        <v>318</v>
+      </c>
+      <c r="C320" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="321" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A321" s="3">
+        <v>36052</v>
+      </c>
+      <c r="B321" s="3" t="s">
+        <v>319</v>
+      </c>
+      <c r="C321" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="322" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A322" s="3">
+        <v>36012</v>
+      </c>
+      <c r="B322" s="3" t="s">
+        <v>320</v>
+      </c>
+      <c r="C322" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="323" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A323" s="3">
+        <v>36008</v>
+      </c>
+      <c r="B323" s="3" t="s">
+        <v>321</v>
+      </c>
+      <c r="C323" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="324" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A324" s="3">
+        <v>35948</v>
+      </c>
+      <c r="B324" s="3" t="s">
+        <v>322</v>
+      </c>
+      <c r="C324" s="2">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:C316"/>
+  <autoFilter ref="A1:C316" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <pageMargins left="0.17" right="0.16" top="0.17" bottom="0.17" header="0.17" footer="0.17"/>
   <pageSetup paperSize="9" orientation="landscape" verticalDpi="0" r:id="rId1"/>
 </worksheet>

</xml_diff>